<commit_message>
Refine D1 publication figures and current-result reporting
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D1 Sensor health/outputs/plot_data/Fig1_D1_dimension_matrix_data.xlsx
+++ b/Project 1 Data Quality Assessment/D1 Sensor health/outputs/plot_data/Fig1_D1_dimension_matrix_data.xlsx
@@ -532,7 +532,8 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>very frequent (&gt;20%)</t>
+          <t>very frequent
+(&gt;20%)</t>
         </is>
       </c>
     </row>
@@ -569,7 +570,8 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>high (sustained)</t>
+          <t>high
+(sustained)</t>
         </is>
       </c>
     </row>
@@ -606,7 +608,8 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>&gt; 3.0 sustained</t>
+          <t>&gt; 3.0
+sustained</t>
         </is>
       </c>
     </row>

</xml_diff>